<commit_message>
fix last sakef verstion
</commit_message>
<xml_diff>
--- a/اسماء شركات الاسنان/دمج الاسمنت.xlsx
+++ b/اسماء شركات الاسنان/دمج الاسمنت.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA3F1813-4A43-4E87-BCC6-42FAA42CDDC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6F28BC7-44B8-49FF-97AB-92FCBE8A0350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18641,16 +18641,22 @@
     <xf numFmtId="1" fontId="11" fillId="6" borderId="7" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="11" fillId="6" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="11" fillId="6" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="11" fillId="6" borderId="5" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="11" fillId="6" borderId="7" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="7" fillId="6" borderId="5" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="11" fillId="6" borderId="5" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="7" fillId="6" borderId="7" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="11" fillId="6" borderId="7" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="11" fillId="0" borderId="5" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -18659,16 +18665,10 @@
     <xf numFmtId="1" fontId="11" fillId="0" borderId="7" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="11" fillId="6" borderId="5" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="7" fillId="6" borderId="5" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="11" fillId="6" borderId="7" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="11" fillId="6" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="11" fillId="6" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="7" fillId="6" borderId="7" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -21435,7 +21435,7 @@
       <c r="A82" s="83">
         <v>55</v>
       </c>
-      <c r="B82" s="93">
+      <c r="B82" s="85">
         <v>1221</v>
       </c>
       <c r="C82" s="31" t="s">
@@ -21452,14 +21452,14 @@
       <c r="H82" s="33">
         <v>23801</v>
       </c>
-      <c r="I82" s="85" t="s">
+      <c r="I82" s="87" t="s">
         <v>4858</v>
       </c>
-      <c r="J82" s="85"/>
+      <c r="J82" s="87"/>
     </row>
     <row r="83" spans="1:12" s="26" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="84"/>
-      <c r="B83" s="94"/>
+      <c r="B83" s="86"/>
       <c r="C83" s="31" t="s">
         <v>4859</v>
       </c>
@@ -21474,8 +21474,8 @@
       <c r="H83" s="33">
         <v>26680</v>
       </c>
-      <c r="I83" s="86"/>
-      <c r="J83" s="86"/>
+      <c r="I83" s="88"/>
+      <c r="J83" s="88"/>
     </row>
     <row r="84" spans="1:12" ht="21.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="4">
@@ -23410,7 +23410,7 @@
       <c r="A148" s="83">
         <v>46</v>
       </c>
-      <c r="B148" s="91">
+      <c r="B148" s="89">
         <v>1542</v>
       </c>
       <c r="C148" s="35" t="s">
@@ -23427,14 +23427,14 @@
       <c r="H148" s="33">
         <v>25461</v>
       </c>
-      <c r="I148" s="85" t="s">
+      <c r="I148" s="87" t="s">
         <v>4858</v>
       </c>
-      <c r="J148" s="85"/>
+      <c r="J148" s="87"/>
     </row>
     <row r="149" spans="1:12" s="26" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="84"/>
-      <c r="B149" s="92"/>
+      <c r="B149" s="90"/>
       <c r="C149" s="35" t="s">
         <v>4914</v>
       </c>
@@ -23449,14 +23449,14 @@
       <c r="H149" s="33">
         <v>28732</v>
       </c>
-      <c r="I149" s="86"/>
-      <c r="J149" s="86"/>
+      <c r="I149" s="88"/>
+      <c r="J149" s="88"/>
     </row>
     <row r="150" spans="1:12" s="26" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="83">
         <v>47</v>
       </c>
-      <c r="B150" s="91">
+      <c r="B150" s="89">
         <v>1545</v>
       </c>
       <c r="C150" s="35" t="s">
@@ -23473,14 +23473,14 @@
       <c r="H150" s="33">
         <v>25339</v>
       </c>
-      <c r="I150" s="85" t="s">
+      <c r="I150" s="87" t="s">
         <v>4858</v>
       </c>
-      <c r="J150" s="85"/>
+      <c r="J150" s="87"/>
     </row>
     <row r="151" spans="1:12" s="26" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="84"/>
-      <c r="B151" s="92"/>
+      <c r="B151" s="90"/>
       <c r="C151" s="35" t="s">
         <v>4917</v>
       </c>
@@ -23495,8 +23495,8 @@
       <c r="H151" s="33">
         <v>26685</v>
       </c>
-      <c r="I151" s="86"/>
-      <c r="J151" s="86"/>
+      <c r="I151" s="88"/>
+      <c r="J151" s="88"/>
     </row>
     <row r="152" spans="1:12" ht="21.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="4">
@@ -54451,7 +54451,7 @@
       <c r="L1163" s="3"/>
     </row>
     <row r="1164" spans="1:12" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A1164" s="87">
+      <c r="A1164" s="93">
         <v>25</v>
       </c>
       <c r="B1164" s="62">
@@ -54473,7 +54473,7 @@
       </c>
     </row>
     <row r="1165" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1165" s="88"/>
+      <c r="A1165" s="94"/>
       <c r="B1165" s="64"/>
       <c r="C1165" s="65" t="s">
         <v>5899</v>
@@ -54494,7 +54494,7 @@
       <c r="A1166" s="83">
         <v>369</v>
       </c>
-      <c r="B1166" s="89">
+      <c r="B1166" s="91">
         <v>99990051</v>
       </c>
       <c r="C1166" s="35" t="s">
@@ -54511,14 +54511,14 @@
       <c r="H1166" s="33">
         <v>28193</v>
       </c>
-      <c r="I1166" s="85" t="s">
+      <c r="I1166" s="87" t="s">
         <v>4750</v>
       </c>
-      <c r="J1166" s="85"/>
+      <c r="J1166" s="87"/>
     </row>
     <row r="1167" spans="1:12" s="26" customFormat="1" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1167" s="84"/>
-      <c r="B1167" s="90"/>
+      <c r="B1167" s="92"/>
       <c r="C1167" s="35" t="s">
         <v>5752</v>
       </c>
@@ -54533,8 +54533,8 @@
       <c r="H1167" s="33">
         <v>28165</v>
       </c>
-      <c r="I1167" s="86"/>
-      <c r="J1167" s="86"/>
+      <c r="I1167" s="88"/>
+      <c r="J1167" s="88"/>
     </row>
     <row r="1168" spans="1:12" ht="21.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1168" s="6">
@@ -54572,7 +54572,7 @@
       <c r="A1169" s="83">
         <v>362</v>
       </c>
-      <c r="B1169" s="89">
+      <c r="B1169" s="91">
         <v>4158</v>
       </c>
       <c r="C1169" s="35" t="s">
@@ -54589,14 +54589,14 @@
       <c r="H1169" s="33">
         <v>34181</v>
       </c>
-      <c r="I1169" s="85" t="s">
+      <c r="I1169" s="87" t="s">
         <v>4858</v>
       </c>
-      <c r="J1169" s="85"/>
+      <c r="J1169" s="87"/>
     </row>
     <row r="1170" spans="1:12" s="26" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1170" s="84"/>
-      <c r="B1170" s="90"/>
+      <c r="B1170" s="92"/>
       <c r="C1170" s="35" t="s">
         <v>5729</v>
       </c>
@@ -54611,14 +54611,14 @@
       <c r="H1170" s="33">
         <v>38060</v>
       </c>
-      <c r="I1170" s="86"/>
-      <c r="J1170" s="86"/>
+      <c r="I1170" s="88"/>
+      <c r="J1170" s="88"/>
     </row>
     <row r="1171" spans="1:12" s="26" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1171" s="83">
         <v>363</v>
       </c>
-      <c r="B1171" s="89">
+      <c r="B1171" s="91">
         <v>4187</v>
       </c>
       <c r="C1171" s="35" t="s">
@@ -54635,14 +54635,14 @@
       <c r="H1171" s="33">
         <v>26827</v>
       </c>
-      <c r="I1171" s="85" t="s">
+      <c r="I1171" s="87" t="s">
         <v>4858</v>
       </c>
-      <c r="J1171" s="85"/>
+      <c r="J1171" s="87"/>
     </row>
     <row r="1172" spans="1:12" s="26" customFormat="1" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1172" s="84"/>
-      <c r="B1172" s="90"/>
+      <c r="B1172" s="92"/>
       <c r="C1172" s="35" t="s">
         <v>5734</v>
       </c>
@@ -54657,8 +54657,8 @@
       <c r="H1172" s="33">
         <v>25598</v>
       </c>
-      <c r="I1172" s="86"/>
-      <c r="J1172" s="86"/>
+      <c r="I1172" s="88"/>
+      <c r="J1172" s="88"/>
     </row>
     <row r="1173" spans="1:12" ht="21.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1173" s="11">
@@ -54792,7 +54792,7 @@
       <c r="A1177" s="83">
         <v>373</v>
       </c>
-      <c r="B1177" s="85" t="s">
+      <c r="B1177" s="87" t="s">
         <v>4750</v>
       </c>
       <c r="C1177" s="35" t="s">
@@ -54809,14 +54809,14 @@
       <c r="H1177" s="33">
         <v>28758</v>
       </c>
-      <c r="I1177" s="85" t="s">
+      <c r="I1177" s="87" t="s">
         <v>4750</v>
       </c>
-      <c r="J1177" s="85"/>
+      <c r="J1177" s="87"/>
     </row>
     <row r="1178" spans="1:12" s="26" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1178" s="84"/>
-      <c r="B1178" s="86"/>
+      <c r="B1178" s="88"/>
       <c r="C1178" s="35" t="s">
         <v>5763</v>
       </c>
@@ -54831,8 +54831,8 @@
       <c r="H1178" s="33">
         <v>35918</v>
       </c>
-      <c r="I1178" s="86"/>
-      <c r="J1178" s="86"/>
+      <c r="I1178" s="88"/>
+      <c r="J1178" s="88"/>
     </row>
     <row r="1179" spans="1:12" ht="21.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1179" s="14">
@@ -55971,24 +55971,6 @@
   </sheetData>
   <autoFilter ref="C1:C1218" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="29">
-    <mergeCell ref="A82:A83"/>
-    <mergeCell ref="B82:B83"/>
-    <mergeCell ref="I82:I83"/>
-    <mergeCell ref="J82:J83"/>
-    <mergeCell ref="A148:A149"/>
-    <mergeCell ref="B148:B149"/>
-    <mergeCell ref="I148:I149"/>
-    <mergeCell ref="J148:J149"/>
-    <mergeCell ref="A150:A151"/>
-    <mergeCell ref="B150:B151"/>
-    <mergeCell ref="I150:I151"/>
-    <mergeCell ref="J150:J151"/>
-    <mergeCell ref="A1171:A1172"/>
-    <mergeCell ref="B1171:B1172"/>
-    <mergeCell ref="I1171:I1172"/>
-    <mergeCell ref="J1171:J1172"/>
-    <mergeCell ref="A1169:A1170"/>
-    <mergeCell ref="B1169:B1170"/>
     <mergeCell ref="A1177:A1178"/>
     <mergeCell ref="B1177:B1178"/>
     <mergeCell ref="I1177:I1178"/>
@@ -56000,6 +55982,24 @@
     <mergeCell ref="B1166:B1167"/>
     <mergeCell ref="I1166:I1167"/>
     <mergeCell ref="J1166:J1167"/>
+    <mergeCell ref="A150:A151"/>
+    <mergeCell ref="B150:B151"/>
+    <mergeCell ref="I150:I151"/>
+    <mergeCell ref="J150:J151"/>
+    <mergeCell ref="A1171:A1172"/>
+    <mergeCell ref="B1171:B1172"/>
+    <mergeCell ref="I1171:I1172"/>
+    <mergeCell ref="J1171:J1172"/>
+    <mergeCell ref="A1169:A1170"/>
+    <mergeCell ref="B1169:B1170"/>
+    <mergeCell ref="A82:A83"/>
+    <mergeCell ref="B82:B83"/>
+    <mergeCell ref="I82:I83"/>
+    <mergeCell ref="J82:J83"/>
+    <mergeCell ref="A148:A149"/>
+    <mergeCell ref="B148:B149"/>
+    <mergeCell ref="I148:I149"/>
+    <mergeCell ref="J148:J149"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>